<commit_message>
Rebuild pipeline for data_final.xlsx (v2.0.0)
- Explicit, reviewable mappings: algorithm synonyms, F2 -> F1 categories,
  method families, WOAH-listed viral diseases with host groups, target groups
- New figures: temporal trend, ML methods, geography and diseases,
  category x disease, disease x stage/theme, reported performance (+ S1)
- Table S1 and mapping QA workbook
- Optional reporting-quality columns with coding rules in template/README.md
- Remove the previous standardisation and figure modules
</commit_message>
<xml_diff>
--- a/template/data_template.xlsx
+++ b/template/data_template.xlsx
@@ -413,58 +413,58 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>ID</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Authors</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Year</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>DOI</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>Journal</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>Disease</t>
-        </is>
-      </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>Algorithm(s)</t>
+          <t>Cat_Algorithms</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Section</t>
+          <t>Algorithms</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
-          <t>Country</t>
+          <t>Countries</t>
         </is>
       </c>
       <c r="J1" t="inlineStr">
         <is>
-          <t>Main metric</t>
+          <t>Diseases</t>
         </is>
       </c>
       <c r="K1" t="inlineStr">
@@ -474,229 +474,375 @@
       </c>
       <c r="L1" t="inlineStr">
         <is>
-          <t>Status</t>
+          <t>Theme</t>
         </is>
       </c>
       <c r="M1" t="inlineStr">
         <is>
+          <t>Target</t>
+        </is>
+      </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Main_Metric_Type</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Main_Metric_Value_min</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>Main_Metric_Value_max</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Sources</t>
+        </is>
+      </c>
+      <c r="S1" t="inlineStr">
+        <is>
+          <t>Validation</t>
+        </is>
+      </c>
+      <c r="T1" t="inlineStr">
+        <is>
+          <t>Reports_AUPRC</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Reports_SensSpec</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
+          <t>Reports_CI</t>
+        </is>
+      </c>
+      <c r="W1" t="inlineStr">
+        <is>
+          <t>Reports_Calibration</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Smith J, Doe A</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Smith John, Doe Anna</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
         <v>2022</v>
       </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>Example: Random Forest for early detection of Disease X in Country Y</t>
-        </is>
-      </c>
       <c r="D2" t="inlineStr">
         <is>
+          <t>Example: Random forest for African swine fever risk mapping</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
           <t>10.xxxx/example.2022.001</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Example Journal of Veterinary Epidemiology</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>Tree Ensemble; Linear Model</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Random Forest; Logistic Regression</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Poland</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
         <is>
           <t>ASF</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
-        <is>
-          <t>Random Forest</t>
-        </is>
-      </c>
-      <c r="H2" t="inlineStr">
-        <is>
-          <t>Outbreak Prediction and Early Warning</t>
-        </is>
-      </c>
-      <c r="I2" t="inlineStr">
-        <is>
-          <t>Poland</t>
-        </is>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>AUC = 0.91</t>
-        </is>
-      </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Surveillance</t>
+          <t>Prediction/Forecasting</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>included</t>
+          <t>Geospatial &amp; Environmental</t>
         </is>
       </c>
       <c r="M2" t="inlineStr">
         <is>
-          <t>Example row - replace with your own extracted data</t>
+          <t>Disease occurrence – animal</t>
         </is>
       </c>
       <c r="N2" t="inlineStr">
         <is>
-          <t>PubMed, Scopus</t>
+          <t>AUC</t>
+        </is>
+      </c>
+      <c r="O2" t="n">
+        <v>0.78</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.91</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>Example row - replace with your own extracted records.</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>PubMed; Scopus</t>
+        </is>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Spatial</t>
+        </is>
+      </c>
+      <c r="T2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>no</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Kowalski M</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>2023</v>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Example: Comparing XGBoost and SVM for FMD risk mapping</t>
-        </is>
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Kowalski Jan</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>2024</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.xxxx/example.2023.002</t>
+          <t>Example: Deep learning host prediction from influenza sequences</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Example Transboundary Diseases Journal</t>
+          <t>10.xxxx/example.2024.002</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>FMD</t>
+          <t>Example Viruses</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>XGBoost, SVM</t>
+          <t>Deep Learning; SVM</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Spatial Epidemiology and Risk Mapping</t>
+          <t>Convolutional Neural Network; Support Vector Machine</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>Thailand, Vietnam</t>
+          <t>Global</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>Accuracy = 87%</t>
+          <t>HPAI; LPAI</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Spatial</t>
+          <t>Other</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>included</t>
+          <t>Emerging Applications and Technologies</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
         <is>
-          <t>Example row - replace with your own extracted data</t>
+          <t>Sequence-based viral trait</t>
         </is>
       </c>
       <c r="N3" t="inlineStr">
         <is>
+          <t>Accuracy</t>
+        </is>
+      </c>
+      <c r="O3" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.96</v>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>Example row - global study (counted in the note under the map, not on it).</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
           <t>WoS</t>
+        </is>
+      </c>
+      <c r="S3" t="inlineStr">
+        <is>
+          <t>Random split/CV</t>
+        </is>
+      </c>
+      <c r="T3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>NA</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Nowak P, Lee K, Garcia R</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Nowak Piotr, Lee Kim</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
         <v>2021</v>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="D4" t="inlineStr">
         <is>
           <t>Example: Systematic review of machine learning in avian influenza surveillance</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="E4" t="inlineStr">
         <is>
           <t>10.xxxx/example.2021.003</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Example One Health Reviews</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Europe; Asia</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
         <is>
           <t>HPAI</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>Methodology/Review</t>
+        </is>
+      </c>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>One Health &amp; Future Perspectives</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
-        <is>
-          <t>Methodological Review</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>International</t>
-        </is>
-      </c>
-      <c r="J4" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="K4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>Review</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
-        <is>
-          <t>excluded</t>
-        </is>
-      </c>
-      <c r="M4" t="inlineStr">
-        <is>
-          <t>Example of an excluded/review record</t>
-        </is>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>PubMed, Scopus, WoS</t>
-        </is>
-      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>Review</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>Example review - excluded from all figures, listed in Table S1.</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>PubMed; Scopus; WoS</t>
+        </is>
+      </c>
+      <c r="S4" t="inlineStr"/>
+      <c r="T4" t="inlineStr"/>
+      <c r="U4" t="inlineStr"/>
+      <c r="V4" t="inlineStr"/>
+      <c r="W4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Use spatial/temporal design columns in Figure 6; map AI and AUPR
- Figure 6C reads Spatial_blocked and Temporal_holdout when present and
  shows counts (k/n) of applicable publications per item
- DISEASE_MAP: 'AI' -> AI; METRIC_SYNONYMS: 'AUPR' -> 'AUPRC'
- Template and coding rules document the two new columns
</commit_message>
<xml_diff>
--- a/template/data_template.xlsx
+++ b/template/data_template.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -514,20 +514,30 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>Spatial_blocked</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
+          <t>Temporal_holdout</t>
+        </is>
+      </c>
+      <c r="V1" t="inlineStr">
+        <is>
           <t>Reports_AUPRC</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>Reports_SensSpec</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>Reports_CI</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>Reports_Calibration</t>
         </is>
@@ -623,20 +633,30 @@
       </c>
       <c r="T2" t="inlineStr">
         <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="U2" t="inlineStr">
+        <is>
           <t>no</t>
         </is>
       </c>
-      <c r="U2" t="inlineStr">
+      <c r="V2" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="W2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="V2" t="inlineStr">
+      <c r="X2" t="inlineStr">
         <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="W2" t="inlineStr">
+      <c r="Y2" t="inlineStr">
         <is>
           <t>no</t>
         </is>
@@ -737,19 +757,25 @@
       </c>
       <c r="U3" t="inlineStr">
         <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
           <t>yes</t>
         </is>
       </c>
-      <c r="V3" t="inlineStr">
+      <c r="X3" t="inlineStr">
         <is>
           <t>no</t>
         </is>
       </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>NA</t>
-        </is>
-      </c>
+      <c r="Y3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -843,6 +869,8 @@
       <c r="U4" t="inlineStr"/>
       <c r="V4" t="inlineStr"/>
       <c r="W4" t="inlineStr"/>
+      <c r="X4" t="inlineStr"/>
+      <c r="Y4" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>